<commit_message>
Updating dataset excel guide to include rental dataset.
</commit_message>
<xml_diff>
--- a/20250815_dataset_guide_MM_V1.xlsx
+++ b/20250815_dataset_guide_MM_V1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\marshall_group\User\gp1mmx\housing_populism\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2316B685-0756-4436-81B7-DDF7FD32AF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77CF363-D218-4B19-B398-20A464525C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5FF58C6B-ED44-4846-AD90-2C48070ED693}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="92">
   <si>
     <t>Dataset</t>
   </si>
@@ -278,18 +278,6 @@
     <t>y</t>
   </si>
   <si>
-    <t>Residential turnover</t>
-  </si>
-  <si>
-    <t>hh_churn_oslaua_2023</t>
-  </si>
-  <si>
-    <t>1997-2022</t>
-  </si>
-  <si>
-    <t>https://data.geods.ac.uk/dataset/residential-mobility-index</t>
-  </si>
-  <si>
     <t>British election survey W22</t>
   </si>
   <si>
@@ -311,22 +299,19 @@
     <t>https://www.britishelectionstudy.com/data-objects/panel-study-data/</t>
   </si>
   <si>
-    <t>Landlord possession claims</t>
-  </si>
-  <si>
-    <t>possession_statistics_2024</t>
-  </si>
-  <si>
-    <t>MAP_CSV</t>
-  </si>
-  <si>
-    <t>https://assets.publishing.service.gov.uk/media/66b360d9a3c2a28abb50de35/Mortgage_and_landlord_statistical_data.zip</t>
-  </si>
-  <si>
-    <t>https://assets.publishing.service.gov.uk/media/620397bce90e077f71cd545b/Mortgage_and_landlord_statistical_data.zip</t>
-  </si>
-  <si>
-    <t>possession_statistics_2021</t>
+    <t>https://www.ons.gov.uk/file?uri=/economy/inflationandpriceindices/datasets/priceindexofprivaterentsukmonthlypricestatistics/21january2026/priceindexofprivaterentsukmonthlypricestatistics.xlsx</t>
+  </si>
+  <si>
+    <t>2015-2025</t>
+  </si>
+  <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>priceindexofprivaterentsukmonthlypricestatistics</t>
+  </si>
+  <si>
+    <t>Rental price</t>
   </si>
 </sst>
 </file>
@@ -1248,33 +1233,33 @@
         <v>79</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D24" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F24" s="1">
-        <v>45897</v>
+        <v>46057</v>
       </c>
       <c r="G24" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
+        <v>80</v>
+      </c>
+      <c r="D25" t="s">
         <v>84</v>
-      </c>
-      <c r="D25" t="s">
-        <v>88</v>
       </c>
       <c r="E25" s="2">
         <v>2021</v>
@@ -1283,18 +1268,18 @@
         <v>45901</v>
       </c>
       <c r="G25" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C26" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E26" s="2">
         <v>2024</v>
@@ -1303,54 +1288,14 @@
         <v>45901</v>
       </c>
       <c r="G26" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>79</v>
-      </c>
-      <c r="B27" t="s">
-        <v>91</v>
-      </c>
-      <c r="C27" t="s">
-        <v>92</v>
-      </c>
-      <c r="D27" t="s">
-        <v>93</v>
-      </c>
-      <c r="E27" s="2">
-        <v>2024</v>
-      </c>
-      <c r="F27" s="1">
-        <v>45902</v>
-      </c>
-      <c r="G27" t="s">
-        <v>94</v>
-      </c>
+      <c r="F27" s="1"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>79</v>
-      </c>
-      <c r="B28" t="s">
-        <v>91</v>
-      </c>
-      <c r="C28" t="s">
-        <v>96</v>
-      </c>
-      <c r="D28" t="s">
-        <v>93</v>
-      </c>
-      <c r="E28" s="2">
-        <v>2021</v>
-      </c>
-      <c r="F28" s="1">
-        <v>45902</v>
-      </c>
-      <c r="G28" t="s">
-        <v>95</v>
-      </c>
+      <c r="F28" s="1"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:G21">

</xml_diff>